<commit_message>
v.2.8.4: sincroniza arquivos de dados de entrada e adiciona gitignore para arquivos temporarios
Versao anterior: v.2.8.3
Nova versao: v.2.8.4

Alteracoes:
- Criado arquivo .gitignore para ignorar arquivos temporarios de bloqueio do Excel/Office (~$*), resolvendo conflitos de permissao no Windows.
- Sincronizados arquivos do diretorio input/ (planilhas de inscricoes e presenca, convocacoes em PDF e exclusao de Figura 14).
- Atualizada a versao para v.2.8.4 nos rodapes e cabecalhos de script.

Validacoes:
- Validacao estatica de sintaxe Node.js em todos os arquivos JS (0 erros).
- Consistencia de versao v.2.8.4 conferida nos rodapes e cabecalhos.
</commit_message>
<xml_diff>
--- a/input/16CTE - Lista de presença (respostas).xlsx
+++ b/input/16CTE - Lista de presença (respostas).xlsx
@@ -1,17 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Antigravity\auto-report-cecate-co\input\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F78067F-1B77-466C-9817-4FD8AC88365A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28680" yWindow="-360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Respostas ao formulário 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Respostas ao formulário 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="126">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -36,16 +58,20 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Telefone </t>
     </r>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
+        <family val="2"/>
       </rPr>
       <t>(XX)XXXXX-XXXX</t>
     </r>
@@ -393,31 +419,68 @@
   </si>
   <si>
     <t>elizangelafreitasdasilva38@gmail.com</t>
+  </si>
+  <si>
+    <t>(64) 993409360</t>
+  </si>
+  <si>
+    <t>Nova Lacerda</t>
+  </si>
+  <si>
+    <t>CACS-FUNDEB</t>
+  </si>
+  <si>
+    <t>Não</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -426,75 +489,69 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="4">
     <dxf>
-      <font/>
       <fill>
-        <patternFill patternType="none"/>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8F9FA"/>
+          <bgColor rgb="FFF8F9FA"/>
+        </patternFill>
       </fill>
-      <border/>
     </dxf>
     <dxf>
-      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF5B3F86"/>
           <bgColor rgb="FF5B3F86"/>
         </patternFill>
       </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8F9FA"/>
-          <bgColor rgb="FFF8F9FA"/>
-        </patternFill>
-      </fill>
-      <border/>
     </dxf>
     <dxf>
       <border>
@@ -514,47 +571,47 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Respostas ao formulário 1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Respostas ao formulário 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:M28" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:M28">
   <tableColumns count="13">
-    <tableColumn name="Carimbo de data/hora" id="1"/>
-    <tableColumn name="Nome Completo:" id="2"/>
-    <tableColumn name="CPF:  XXX.XXX.XXX-XX" id="3"/>
-    <tableColumn name="Telefone: (DD)XXXXX-XXXX" id="4"/>
-    <tableColumn name="E-mail: xxxxxxx@xxxmail.com" id="5"/>
-    <tableColumn name="Você já está inscrito no Curso de Capacitação em Transporte Escolar?" id="6"/>
-    <tableColumn name="Data de Nascimento" id="7"/>
-    <tableColumn name="Telefone (XX)XXXXX-XXXX" id="8"/>
-    <tableColumn name="Município que representa:" id="9"/>
-    <tableColumn name="Você faz parte do:" id="10"/>
-    <tableColumn name="Que cargo você ocupa na gestão municipal?" id="11"/>
-    <tableColumn name="Prezado(a) Gestor(a), _x000a__x000a_Se existe algum caso de sucesso da gestão do transporte escolar no seu município, gostaríamos conhecer mais um pouco ao respeito._x000a__x000a_Por favor, relate de forma sucinta o caso de sucesso no espaço a seguir:" id="12"/>
-    <tableColumn name="Que cargo você ocupa no CACS-FUNDEB?" id="13"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Carimbo de data/hora"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nome Completo:"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="CPF:  XXX.XXX.XXX-XX"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Telefone: (DD)XXXXX-XXXX"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="E-mail: xxxxxxx@xxxmail.com"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Você já está inscrito no Curso de Capacitação em Transporte Escolar?"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Data de Nascimento"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Telefone (XX)XXXXX-XXXX"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Município que representa:"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Você faz parte do:"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Que cargo você ocupa na gestão municipal?"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Prezado(a) Gestor(a), _x000a__x000a_Se existe algum caso de sucesso da gestão do transporte escolar no seu município, gostaríamos conhecer mais um pouco ao respeito._x000a__x000a_Por favor, relate de forma sucinta o caso de sucesso no espaço a seguir:"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Que cargo você ocupa no CACS-FUNDEB?"/>
   </tableColumns>
-  <tableStyleInfo name="Respostas ao formulário 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Respostas ao formulário 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -744,33 +801,36 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:M28"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.25"/>
-    <col customWidth="1" min="2" max="2" width="18.88"/>
-    <col customWidth="1" min="3" max="3" width="22.13"/>
-    <col customWidth="1" min="4" max="4" width="25.38"/>
-    <col customWidth="1" min="5" max="5" width="27.0"/>
-    <col customWidth="1" min="6" max="6" width="37.63"/>
-    <col customWidth="1" min="7" max="7" width="20.13"/>
-    <col customWidth="1" min="8" max="8" width="24.88"/>
-    <col customWidth="1" min="9" max="9" width="24.13"/>
-    <col customWidth="1" min="10" max="10" width="18.88"/>
-    <col customWidth="1" min="11" max="11" width="37.25"/>
-    <col customWidth="1" min="12" max="12" width="37.63"/>
-    <col customWidth="1" min="13" max="13" width="35.63"/>
-    <col customWidth="1" min="14" max="19" width="18.88"/>
+    <col min="1" max="1" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
+    <col min="6" max="6" width="37.5703125" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
+    <col min="9" max="9" width="24.140625" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="37.28515625" customWidth="1"/>
+    <col min="12" max="12" width="37.5703125" customWidth="1"/>
+    <col min="13" max="13" width="35.5703125" customWidth="1"/>
+    <col min="14" max="19" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -811,9 +871,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
-        <v>46196.37921359953</v>
+        <v>46196.379213599532</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>13</v>
@@ -828,19 +888,27 @@
         <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
+        <v>125</v>
+      </c>
+      <c r="G2" s="5">
+        <v>35481</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+    </row>
+    <row r="3" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
-        <v>46196.38637827546</v>
+        <v>46196.386378275463</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>18</v>
@@ -857,17 +925,17 @@
       <c r="F3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+    </row>
+    <row r="4" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>46196.38720524305</v>
+        <v>46196.387205243052</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>22</v>
@@ -884,17 +952,17 @@
       <c r="F4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
+      <c r="G4" s="4"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+    </row>
+    <row r="5" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
-        <v>46196.38786930556</v>
+        <v>46196.387869305559</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>26</v>
@@ -911,17 +979,17 @@
       <c r="F5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+    </row>
+    <row r="6" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
-        <v>46196.39124025463</v>
+        <v>46196.391240254627</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>30</v>
@@ -938,15 +1006,15 @@
       <c r="F6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+    </row>
+    <row r="7" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>46196.391299571755</v>
       </c>
@@ -965,17 +1033,17 @@
       <c r="F7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+    </row>
+    <row r="8" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>46196.3926847338</v>
+        <v>46196.392684733801</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>38</v>
@@ -992,17 +1060,17 @@
       <c r="F8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+    </row>
+    <row r="9" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>46196.39356967593</v>
+        <v>46196.393569675929</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>42</v>
@@ -1017,19 +1085,27 @@
         <v>45</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
+        <v>125</v>
+      </c>
+      <c r="G9" s="5">
+        <v>35481</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+    </row>
+    <row r="10" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>46196.39360574074</v>
+        <v>46196.393605740741</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>46</v>
@@ -1046,17 +1122,17 @@
       <c r="F10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-    </row>
-    <row r="11" ht="22.5" customHeight="1">
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+    </row>
+    <row r="11" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>46196.39367449074</v>
+        <v>46196.393674490741</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>50</v>
@@ -1073,17 +1149,17 @@
       <c r="F11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+    </row>
+    <row r="12" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>46196.39419168982</v>
+        <v>46196.394191689818</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>54</v>
@@ -1100,15 +1176,15 @@
       <c r="F12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-    </row>
-    <row r="13" ht="22.5" customHeight="1">
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+    </row>
+    <row r="13" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>46196.397766435184</v>
       </c>
@@ -1127,17 +1203,17 @@
       <c r="F13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-    </row>
-    <row r="14" ht="22.5" customHeight="1">
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+    </row>
+    <row r="14" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>46196.39947160879</v>
+        <v>46196.399471608791</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>62</v>
@@ -1154,15 +1230,15 @@
       <c r="F14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+    </row>
+    <row r="15" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>46196.414961365736</v>
       </c>
@@ -1181,15 +1257,15 @@
       <c r="F15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-    </row>
-    <row r="16" ht="22.5" customHeight="1">
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+    </row>
+    <row r="16" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>46197.390446562495</v>
       </c>
@@ -1208,17 +1284,17 @@
       <c r="F16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+    </row>
+    <row r="17" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
-        <v>46197.39147766204</v>
+        <v>46197.391477662037</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>74</v>
@@ -1235,15 +1311,15 @@
       <c r="F17" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+    </row>
+    <row r="18" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>46197.39210730324</v>
       </c>
@@ -1262,15 +1338,15 @@
       <c r="F18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+    </row>
+    <row r="19" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>46197.392847256946</v>
       </c>
@@ -1289,15 +1365,15 @@
       <c r="F19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+    </row>
+    <row r="20" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>46197.392916909725</v>
       </c>
@@ -1316,17 +1392,17 @@
       <c r="F20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+    </row>
+    <row r="21" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
-        <v>46197.39298415509</v>
+        <v>46197.392984155093</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>90</v>
@@ -1343,17 +1419,17 @@
       <c r="F21" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+    </row>
+    <row r="22" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
-        <v>46197.39321525463</v>
+        <v>46197.393215254633</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>94</v>
@@ -1370,17 +1446,17 @@
       <c r="F22" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+    </row>
+    <row r="23" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>46197.393380625</v>
+        <v>46197.393380624999</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>98</v>
@@ -1397,17 +1473,17 @@
       <c r="F23" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+    </row>
+    <row r="24" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
-        <v>46197.39372945602</v>
+        <v>46197.393729456016</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>102</v>
@@ -1424,17 +1500,17 @@
       <c r="F24" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+    </row>
+    <row r="25" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
-        <v>46197.39434576389</v>
+        <v>46197.394345763889</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>106</v>
@@ -1451,17 +1527,17 @@
       <c r="F25" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-    </row>
-    <row r="26" ht="22.5" customHeight="1">
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+    </row>
+    <row r="26" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
-        <v>46197.4343233449</v>
+        <v>46197.434323344904</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>110</v>
@@ -1478,15 +1554,15 @@
       <c r="F26" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
-    </row>
-    <row r="27" ht="22.5" customHeight="1">
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+    </row>
+    <row r="27" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>46197.504957453704</v>
       </c>
@@ -1503,19 +1579,27 @@
         <v>117</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
+        <v>125</v>
+      </c>
+      <c r="G27" s="5">
+        <v>35481</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+    </row>
+    <row r="28" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
-        <v>46197.52073636574</v>
+        <v>46197.520736365739</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>118</v>
@@ -1532,18 +1616,18 @@
       <c r="F28" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>